<commit_message>
page update & db update
</commit_message>
<xml_diff>
--- a/TPNelem.xlsx
+++ b/TPNelem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AKIE01-2022\Python_script\DIサイト\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AKIE01-2025\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A37446-B278-4E65-A135-2CBAC023EAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC1F8E4-F347-491B-A720-F6B52A743608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32790" yWindow="420" windowWidth="23775" windowHeight="15180" activeTab="2" xr2:uid="{A8DE39AC-9138-4E02-B691-3AB8BC6B522D}"/>
+    <workbookView xWindow="34560" yWindow="960" windowWidth="22845" windowHeight="13215" activeTab="2" xr2:uid="{A8DE39AC-9138-4E02-B691-3AB8BC6B522D}"/>
   </bookViews>
   <sheets>
     <sheet name="DB" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="elem" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">elem!$A$1:$L$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">elem!$A$1:$L$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="110">
   <si>
     <t>K（mEq）</t>
     <phoneticPr fontId="1"/>
@@ -1057,6 +1057,21 @@
   </si>
   <si>
     <t>補液｜ソリタ-T3号輸液</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ヴィーンD輸液</t>
+    <rPh sb="5" eb="7">
+      <t>ユエキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ヴィーンD輸液</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>補液｜ヴィーンD輸液</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1215,15 +1230,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:colOff>933450</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>19869</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>114845</xdr:rowOff>
+      <xdr:colOff>267519</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>162470</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1246,7 +1261,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8677275" y="10020300"/>
+          <a:off x="8924925" y="12211050"/>
           <a:ext cx="5868219" cy="3905795"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1260,9 +1275,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 テーマ">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1300,7 +1315,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1406,7 +1421,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1548,7 +1563,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1556,7 +1571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ED4D603-50C3-490D-BFA1-F7765C4DA5D3}">
-  <dimension ref="A1:T45"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="34.5" customWidth="1"/>
@@ -3973,7 +3988,7 @@
         <v>0</v>
       </c>
       <c r="O39" s="6">
-        <f t="shared" si="13"/>
+        <f>H39/F39</f>
         <v>113.23584905660377</v>
       </c>
       <c r="P39">
@@ -4203,7 +4218,7 @@
         <v>292.2</v>
       </c>
       <c r="T43" s="10">
-        <f t="shared" ref="T43" si="20">P43+R43</f>
+        <f t="shared" ref="T43:T45" si="20">P43+R43</f>
         <v>246.60000000000002</v>
       </c>
     </row>
@@ -4289,8 +4304,72 @@
         <v>1500.1879999999999</v>
       </c>
       <c r="T45" s="10">
-        <f>H45/F45</f>
-        <v>300.21929824561408</v>
+        <f>P45+R45</f>
+        <v>1368.8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20">
+      <c r="A46" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" s="2">
+        <v>500</v>
+      </c>
+      <c r="C46" s="2">
+        <v>25</v>
+      </c>
+      <c r="D46" s="2">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2">
+        <v>0</v>
+      </c>
+      <c r="G46" s="2">
+        <v>100</v>
+      </c>
+      <c r="H46" s="2">
+        <v>100</v>
+      </c>
+      <c r="I46" s="2">
+        <v>65</v>
+      </c>
+      <c r="J46" s="2">
+        <v>2</v>
+      </c>
+      <c r="K46" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="L46" s="2">
+        <v>0</v>
+      </c>
+      <c r="M46" s="2">
+        <v>1</v>
+      </c>
+      <c r="O46" s="6" t="e">
+        <f>H46/F46</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="P46" s="10">
+        <f>C46*4</f>
+        <v>100</v>
+      </c>
+      <c r="Q46" s="10">
+        <f>D46*4</f>
+        <v>0</v>
+      </c>
+      <c r="R46">
+        <v>0</v>
+      </c>
+      <c r="S46" s="10">
+        <f>SUM(P46:R46)</f>
+        <v>100</v>
+      </c>
+      <c r="T46" s="10">
+        <f>P46+R46</f>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -4305,7 +4384,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDC7C856-4D92-4C40-A383-D2F62D797670}">
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="34.5" customWidth="1"/>
@@ -5993,6 +6072,44 @@
         <v>5.7142857142857143E-3</v>
       </c>
     </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46">
+        <v>0.05</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0.2</v>
+      </c>
+      <c r="H46">
+        <v>0.2</v>
+      </c>
+      <c r="I46">
+        <v>0.13</v>
+      </c>
+      <c r="J46">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="K46">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="L46">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <dataConsolidate/>
   <phoneticPr fontId="1"/>
@@ -6003,7 +6120,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EB05657-7C92-4504-9151-023EF147012E}">
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="34.5" customWidth="1"/>
@@ -7268,434 +7385,472 @@
       <c r="M32" s="8"/>
     </row>
     <row r="33" spans="1:13">
-      <c r="A33" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B33" s="8">
-        <v>1</v>
-      </c>
-      <c r="C33" s="8">
-        <v>0.1575</v>
-      </c>
-      <c r="D33" s="8">
-        <v>6.7500000000000004E-2</v>
-      </c>
-      <c r="E33" s="8">
-        <v>1.8500000000000003E-2</v>
-      </c>
-      <c r="F33" s="8">
-        <v>1.0800000000000001E-2</v>
-      </c>
-      <c r="G33" s="8">
-        <v>1.0649999999999999</v>
-      </c>
-      <c r="H33" s="8">
-        <v>0.7965000000000001</v>
-      </c>
-      <c r="I33" s="8">
-        <v>8.5000000000000006E-3</v>
-      </c>
-      <c r="J33" s="8">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="K33" s="8">
-        <v>1.455E-2</v>
-      </c>
-      <c r="L33" s="8">
-        <v>8.3000000000000001E-3</v>
-      </c>
-      <c r="M33" s="8"/>
+      <c r="A33" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>0.05</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0.2</v>
+      </c>
+      <c r="H33">
+        <v>0.2</v>
+      </c>
+      <c r="I33">
+        <v>0.13</v>
+      </c>
+      <c r="J33">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="K33">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="8" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B34" s="8">
         <v>1</v>
       </c>
       <c r="C34" s="8">
-        <v>0.21224000000000001</v>
+        <v>0.1575</v>
       </c>
       <c r="D34" s="8">
-        <v>6.4000000000000001E-2</v>
+        <v>6.7500000000000004E-2</v>
       </c>
       <c r="E34" s="8">
-        <v>5.1520000000000003E-2</v>
+        <v>1.8500000000000003E-2</v>
       </c>
       <c r="F34" s="8">
-        <v>0.01</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="G34" s="8">
-        <v>1.6</v>
+        <v>1.0649999999999999</v>
       </c>
       <c r="H34" s="8">
-        <v>1.31264</v>
+        <v>0.7965000000000001</v>
       </c>
       <c r="I34" s="8">
-        <v>6.2399999999999997E-2</v>
+        <v>8.5000000000000006E-3</v>
       </c>
       <c r="J34" s="8">
-        <v>7.5200000000000003E-2</v>
+        <v>2.7099999999999999E-2</v>
       </c>
       <c r="K34" s="8">
-        <v>7.1199999999999999E-2</v>
+        <v>1.455E-2</v>
       </c>
       <c r="L34" s="8">
-        <v>5.4399999999999997E-2</v>
+        <v>8.3000000000000001E-3</v>
       </c>
       <c r="M34" s="8"/>
     </row>
     <row r="35" spans="1:13">
       <c r="A35" s="8" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B35" s="8">
         <v>1</v>
       </c>
       <c r="C35" s="8">
-        <v>0.15840000000000001</v>
+        <v>0.21224000000000001</v>
       </c>
       <c r="D35" s="8">
-        <v>5.3999999999999999E-2</v>
+        <v>6.4000000000000001E-2</v>
       </c>
       <c r="E35" s="8">
-        <v>3.8399999999999997E-2</v>
+        <v>5.1520000000000003E-2</v>
       </c>
       <c r="F35" s="8">
-        <v>8.4399999999999996E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G35" s="8">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="H35" s="8">
-        <v>0.97920000000000007</v>
+        <v>1.31264</v>
       </c>
       <c r="I35" s="8">
-        <v>0.04</v>
+        <v>6.2399999999999997E-2</v>
       </c>
       <c r="J35" s="8">
-        <v>3.0800000000000001E-2</v>
+        <v>7.5200000000000003E-2</v>
       </c>
       <c r="K35" s="8">
-        <v>5.8000000000000003E-2</v>
+        <v>7.1199999999999999E-2</v>
       </c>
       <c r="L35" s="8">
-        <v>1.72E-2</v>
+        <v>5.4399999999999997E-2</v>
       </c>
       <c r="M35" s="8"/>
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B36" s="8">
         <v>1</v>
       </c>
       <c r="C36" s="8">
-        <v>0.21133333333333332</v>
+        <v>0.15840000000000001</v>
       </c>
       <c r="D36" s="8">
-        <v>4.7E-2</v>
+        <v>5.3999999999999999E-2</v>
       </c>
       <c r="E36" s="8">
-        <v>1.7000000000000001E-3</v>
+        <v>3.8399999999999997E-2</v>
       </c>
       <c r="F36" s="8">
-        <v>6.6666666666666671E-3</v>
+        <v>8.4399999999999996E-3</v>
       </c>
       <c r="G36" s="8">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="H36" s="8">
-        <v>0.86033333333333339</v>
+        <v>0.97920000000000007</v>
       </c>
       <c r="I36" s="8">
-        <v>3.7666666666666668E-2</v>
+        <v>0.04</v>
       </c>
       <c r="J36" s="8">
-        <v>1.8499999999999999E-2</v>
+        <v>3.0800000000000001E-2</v>
       </c>
       <c r="K36" s="8">
-        <v>4.306666666666667E-2</v>
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="L36" s="8">
-        <v>1.0966666666666666E-2</v>
+        <v>1.72E-2</v>
       </c>
       <c r="M36" s="8"/>
     </row>
     <row r="37" spans="1:13">
       <c r="A37" s="8" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B37" s="8">
         <v>1</v>
       </c>
       <c r="C37" s="8">
-        <v>0.20599999999999999</v>
+        <v>0.21133333333333332</v>
       </c>
       <c r="D37" s="8">
-        <v>5.28E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="E37" s="8">
-        <v>5.28E-2</v>
+        <v>1.7000000000000001E-3</v>
       </c>
       <c r="F37" s="8">
-        <v>8.2799999999999992E-3</v>
+        <v>6.6666666666666671E-3</v>
       </c>
       <c r="G37" s="8">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H37" s="8">
-        <v>1.2992000000000001</v>
+        <v>0.86033333333333339</v>
       </c>
       <c r="I37" s="8">
-        <v>5.1999999999999998E-2</v>
+        <v>3.7666666666666668E-2</v>
       </c>
       <c r="J37" s="8">
-        <v>5.7200000000000001E-2</v>
+        <v>1.8499999999999999E-2</v>
       </c>
       <c r="K37" s="8">
-        <v>0.04</v>
+        <v>4.306666666666667E-2</v>
       </c>
       <c r="L37" s="8">
-        <v>2.4799999999999999E-2</v>
+        <v>1.0966666666666666E-2</v>
       </c>
       <c r="M37" s="8"/>
     </row>
     <row r="38" spans="1:13">
       <c r="A38" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B38" s="8">
+        <v>1</v>
+      </c>
+      <c r="C38" s="8">
+        <v>0.20599999999999999</v>
+      </c>
+      <c r="D38" s="8">
+        <v>5.28E-2</v>
+      </c>
+      <c r="E38" s="8">
+        <v>5.28E-2</v>
+      </c>
+      <c r="F38" s="8">
+        <v>8.2799999999999992E-3</v>
+      </c>
+      <c r="G38" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="H38" s="8">
+        <v>1.2992000000000001</v>
+      </c>
+      <c r="I38" s="8">
+        <v>5.1999999999999998E-2</v>
+      </c>
+      <c r="J38" s="8">
+        <v>5.7200000000000001E-2</v>
+      </c>
+      <c r="K38" s="8">
+        <v>0.04</v>
+      </c>
+      <c r="L38" s="8">
+        <v>2.4799999999999999E-2</v>
+      </c>
+      <c r="M38" s="8"/>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B38" s="8">
-        <v>1</v>
-      </c>
-      <c r="C38" s="8">
+      <c r="B39" s="8">
+        <v>1</v>
+      </c>
+      <c r="C39" s="8">
         <v>0.15620000000000001</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D39" s="8">
         <v>4.3799999999999999E-2</v>
       </c>
-      <c r="E38" s="8">
+      <c r="E39" s="8">
         <v>2.23E-2</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F39" s="8">
         <v>6.8999999999999999E-3</v>
       </c>
-      <c r="G38" s="8">
-        <v>1</v>
-      </c>
-      <c r="H38" s="8">
+      <c r="G39" s="8">
+        <v>1</v>
+      </c>
+      <c r="H39" s="8">
         <v>0.82550000000000001</v>
       </c>
-      <c r="I38" s="8">
+      <c r="I39" s="8">
         <v>3.2000000000000001E-2</v>
       </c>
-      <c r="J38" s="8">
+      <c r="J39" s="8">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="K38" s="8">
+      <c r="K39" s="8">
         <v>2.2000000000000002E-2</v>
       </c>
-      <c r="L38" s="8">
+      <c r="L39" s="8">
         <v>1.6E-2</v>
       </c>
-      <c r="M38" s="8"/>
-    </row>
-    <row r="39" spans="1:13">
-      <c r="A39" t="s">
+      <c r="M39" s="8"/>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" t="s">
         <v>103</v>
       </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
-      <c r="C39">
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40">
         <v>0.13750000000000001</v>
       </c>
-      <c r="D39">
+      <c r="D40">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="E39">
+      <c r="E40">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="F39">
+      <c r="F40">
         <v>7.0666666666666673E-3</v>
       </c>
-      <c r="G39">
-        <v>1</v>
-      </c>
-      <c r="H39">
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
         <v>0.80020000000000002</v>
       </c>
-      <c r="I39">
+      <c r="I40">
         <v>5.6956521739130433E-2</v>
       </c>
-      <c r="J39">
+      <c r="J40">
         <v>4.7058823529411764E-2</v>
       </c>
-      <c r="K39">
+      <c r="K40">
         <v>4.8778054862842882E-2</v>
       </c>
-      <c r="L39">
+      <c r="L40">
         <v>3.3909465020576131E-2</v>
       </c>
-      <c r="M39" s="8"/>
-    </row>
-    <row r="40" spans="1:13">
-      <c r="A40" s="8" t="s">
+      <c r="M40" s="8"/>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B40" s="8">
-        <v>1</v>
-      </c>
-      <c r="C40" s="8">
+      <c r="B41" s="8">
+        <v>1</v>
+      </c>
+      <c r="C41" s="8">
         <v>0.15620000000000001</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D41" s="8">
         <v>4.3799999999999999E-2</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E41" s="8">
         <v>2.23E-2</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F41" s="8">
         <v>6.8999999999999999E-3</v>
       </c>
-      <c r="G40" s="8">
-        <v>1</v>
-      </c>
-      <c r="H40" s="8">
+      <c r="G41" s="8">
+        <v>1</v>
+      </c>
+      <c r="H41" s="8">
         <v>0.82550000000000001</v>
       </c>
-      <c r="I40" s="8">
+      <c r="I41" s="8">
         <v>3.2000000000000001E-2</v>
       </c>
-      <c r="J40" s="8">
+      <c r="J41" s="8">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="K40" s="8">
+      <c r="K41" s="8">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="L40" s="8">
+      <c r="L41" s="8">
         <v>1.6E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13">
-      <c r="A41" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B41">
-        <v>1</v>
-      </c>
-      <c r="C41">
-        <v>0.1875</v>
-      </c>
-      <c r="D41">
-        <v>5.2499999999999998E-2</v>
-      </c>
-      <c r="E41">
-        <v>0.06</v>
-      </c>
-      <c r="F41">
-        <v>8.6E-3</v>
-      </c>
-      <c r="G41">
-        <v>1.5</v>
-      </c>
-      <c r="H41">
-        <v>1.29</v>
-      </c>
-      <c r="I41">
-        <v>9.3260869565217383E-2</v>
-      </c>
-      <c r="J41">
-        <v>4.0920716112531973E-2</v>
-      </c>
-      <c r="K41">
-        <v>5.2369077306733167E-2</v>
-      </c>
-      <c r="L41">
-        <v>3.9506172839506172E-2</v>
       </c>
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42">
-        <v>0.13200000000000001</v>
+        <v>0.1875</v>
       </c>
       <c r="D42">
-        <v>9.5000000000000001E-2</v>
+        <v>5.2499999999999998E-2</v>
       </c>
       <c r="E42">
-        <v>6.6000000000000003E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F42">
-        <v>1.5162162162162162E-2</v>
+        <v>8.6E-3</v>
       </c>
       <c r="G42">
         <v>1.5</v>
       </c>
       <c r="H42">
-        <v>1.1220000000000001</v>
+        <v>1.29</v>
       </c>
       <c r="I42">
-        <v>0.11434782608695652</v>
+        <v>9.3260869565217383E-2</v>
       </c>
       <c r="J42">
-        <v>5.9335038363171354E-2</v>
+        <v>4.0920716112531973E-2</v>
       </c>
       <c r="K42">
-        <v>5.0374064837905241E-2</v>
+        <v>5.2369077306733167E-2</v>
       </c>
       <c r="L42">
-        <v>2.6337448559670781E-2</v>
+        <v>3.9506172839506172E-2</v>
       </c>
     </row>
     <row r="43" spans="1:13">
       <c r="A43" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43">
-        <v>0.153</v>
+        <v>0.13200000000000001</v>
       </c>
       <c r="D43">
-        <v>5.7000000000000002E-2</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="E43">
-        <v>6.9000000000000006E-2</v>
+        <v>6.6000000000000003E-2</v>
       </c>
       <c r="F43">
-        <v>8.8071428571428571E-3</v>
+        <v>1.5162162162162162E-2</v>
       </c>
       <c r="G43">
         <v>1.5</v>
       </c>
       <c r="H43">
+        <v>1.1220000000000001</v>
+      </c>
+      <c r="I43">
+        <v>0.11434782608695652</v>
+      </c>
+      <c r="J43">
+        <v>5.9335038363171354E-2</v>
+      </c>
+      <c r="K43">
+        <v>5.0374064837905241E-2</v>
+      </c>
+      <c r="L43">
+        <v>2.6337448559670781E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44">
+        <v>0.153</v>
+      </c>
+      <c r="D44">
+        <v>5.7000000000000002E-2</v>
+      </c>
+      <c r="E44">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="F44">
+        <v>8.8071428571428571E-3</v>
+      </c>
+      <c r="G44">
+        <v>1.5</v>
+      </c>
+      <c r="H44">
         <v>1.2329999999999999</v>
       </c>
-      <c r="I43">
+      <c r="I44">
         <v>1.9565217391304349E-2</v>
       </c>
-      <c r="J43">
+      <c r="J44">
         <v>1.0230179028132993E-2</v>
       </c>
-      <c r="K43">
+      <c r="K44">
         <v>1.8703241895261843E-2</v>
       </c>
-      <c r="L43">
+      <c r="L44">
         <v>1.3168724279835391E-2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L40" xr:uid="{9EB05657-7C92-4504-9151-023EF147012E}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L40">
-      <sortCondition ref="A2:A40" customList="総合,蛋白,糖質,電解,補液,経口"/>
+  <autoFilter ref="A1:L41" xr:uid="{9EB05657-7C92-4504-9151-023EF147012E}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L41">
+      <sortCondition ref="A2:A41" customList="総合,蛋白,糖質,電解,補液,経口"/>
     </sortState>
   </autoFilter>
   <dataConsolidate/>

</xml_diff>